<commit_message>
WIP: algorithm family_vN versioning, tune CLI, and two-step train UI.
Keep official release at v0.3.0; exclude incomplete hyperparam tune artifacts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/reports/comparison/feature_importance_top10_all.xlsx
+++ b/outputs/reports/comparison/feature_importance_top10_all.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="전체TOP10(all)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="catboost" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="easy_ensemble" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="gradient_boosting" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="random_forest" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="stacked_ensemble" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체TOP10(all)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="catboost_v1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="easy_ensemble_v1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gradient_boosting_v1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="random_forest_v1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stacked_ensemble_v1" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,24 +469,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>부서코드</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.06671461789117154</v>
+        <v>0.0720834366819162</v>
       </c>
       <c r="F2" t="n">
-        <v>6.671461789117155</v>
+        <v>7.208343668191625</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -495,7 +495,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.67%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=7.21%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -505,24 +505,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.06495441989195058</v>
+        <v>0.06054513955043873</v>
       </c>
       <c r="F3" t="n">
-        <v>6.495441989195059</v>
+        <v>6.054513955043876</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.50%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.05%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -541,24 +541,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>기관유형코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.05547755973096497</v>
+        <v>0.05896145497730271</v>
       </c>
       <c r="F4" t="n">
-        <v>5.547755973096498</v>
+        <v>5.896145497730275</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=5.55%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=5.90%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -577,24 +577,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>LAF_CPRN_AID_BIZCT_RT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>보조사업자설립년수</t>
+          <t>지자체대비보조사업금액비율</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.05417814811546744</v>
+        <v>0.05096941996978932</v>
       </c>
       <c r="F5" t="n">
-        <v>5.417814811546745</v>
+        <v>5.096941996978935</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -603,7 +603,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=5.42%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 지자체대비보조사업금액비율(LAF_CPRN_AID_BIZCT_RT). 기여도(정규화 비중)=5.10%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -613,24 +613,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RPRSV_AGGP_DV_CD</t>
+          <t>SECT_CD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대표자연령대구분코드</t>
+          <t>부문코드</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.05058522443296955</v>
+        <v>0.04933380106314258</v>
       </c>
       <c r="F6" t="n">
-        <v>5.058522443296956</v>
+        <v>4.933380106314261</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=5.06%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=4.93%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -649,24 +649,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>대표자연령대구분코드</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.04458071949171321</v>
+        <v>0.04914549675775322</v>
       </c>
       <c r="F7" t="n">
-        <v>4.458071949171321</v>
+        <v>4.914549675775325</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=4.46%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=4.91%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -685,24 +685,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>INST_TY_CD</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>기관유형코드</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.04060187085898578</v>
+        <v>0.04751753225903853</v>
       </c>
       <c r="F8" t="n">
-        <v>4.060187085898579</v>
+        <v>4.751753225903856</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=4.06%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=4.75%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -721,24 +721,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>지방자치단체코드</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.03611816776722611</v>
+        <v>0.04720868290349021</v>
       </c>
       <c r="F9" t="n">
-        <v>3.611816776722611</v>
+        <v>4.720868290349023</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=3.61%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.72%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -757,24 +757,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SECT_CD</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>부문코드</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.03477271178468273</v>
+        <v>0.04484785765179874</v>
       </c>
       <c r="F10" t="n">
-        <v>3.477271178468274</v>
+        <v>4.484785765179876</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -783,7 +783,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.48%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=4.48%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -793,24 +793,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LBST_PLAN_RT</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>인건비계획비율</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.0344039068366</v>
+        <v>0.03747459357124595</v>
       </c>
       <c r="F11" t="n">
-        <v>3.44039068366</v>
+        <v>3.747459357124598</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>변수 의미: 인건비계획비율(LBST_PLAN_RT). 기여도(정규화 비중)=3.44%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=3.75%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -829,24 +829,24 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MBR_NUM</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>회원수</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.1027335695024538</v>
+        <v>0.1781127861529395</v>
       </c>
       <c r="F12" t="n">
-        <v>0.006969778495202472</v>
+        <v>0.0008332288532263421</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=10.27%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=17.81%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -865,24 +865,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>기관유형코드</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.09652091154231966</v>
+        <v>0.09715242881070832</v>
       </c>
       <c r="F13" t="n">
-        <v>0.006548291633037551</v>
+        <v>0.0004544884653962522</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=9.65%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=9.72%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -901,24 +901,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>MBR_NUM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>회원수</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.07809443240098939</v>
+        <v>0.09659408151866568</v>
       </c>
       <c r="F14" t="n">
-        <v>0.005298179535467795</v>
+        <v>0.0004518764627214344</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=7.81%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=9.66%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -937,24 +937,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BIZ_MDCN</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>사업개월수</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.06968751652302239</v>
+        <v>0.08096035734221936</v>
       </c>
       <c r="F15" t="n">
-        <v>0.00472782710070857</v>
+        <v>0.0003787403878300344</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>변수 의미: 사업개월수(BIZ_MDCN). 기여도(정규화 비중)=6.97%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=8.10%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -973,24 +973,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LAF_PFM_AID_BIZ_NUM</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>지자체수행보조사업수</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.05950933220535835</v>
+        <v>0.07146845337799287</v>
       </c>
       <c r="F16" t="n">
-        <v>0.004037306071204505</v>
+        <v>0.0003343363423604639</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -999,7 +999,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>변수 의미: 지자체수행보조사업수(LAF_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=5.95%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=7.15%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1009,24 +1009,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>당해년도수행보조사업수</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.05448633215248471</v>
+        <v>0.04578447794526556</v>
       </c>
       <c r="F17" t="n">
-        <v>0.003696529459241427</v>
+        <v>0.0002141842193246202</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=5.45%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.58%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1045,24 +1045,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.04909321630624239</v>
+        <v>0.03852596314907911</v>
       </c>
       <c r="F18" t="n">
-        <v>0.003330642991660082</v>
+        <v>0.0001802281845537101</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=4.91%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=3.85%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1081,24 +1081,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LBST_PLAN_RT</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>인건비계획비율</t>
+          <t>대표자연령대구분코드</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.04446676888912223</v>
+        <v>0.03740926856505316</v>
       </c>
       <c r="F19" t="n">
-        <v>0.003016769796430951</v>
+        <v>0.0001750041792043522</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>변수 의미: 인건비계획비율(LBST_PLAN_RT). 기여도(정규화 비중)=4.45%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=3.74%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1117,24 +1117,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BIZCT_PYHWY_AMT</t>
+          <t>LAF_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>사업비자부담금액</t>
+          <t>지자체수행보조사업수</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.03666790038597665</v>
+        <v>0.03629257398101535</v>
       </c>
       <c r="F20" t="n">
-        <v>0.002487669267330406</v>
+        <v>0.0001697801738549387</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>변수 의미: 사업비자부담금액(BIZCT_PYHWY_AMT). 기여도(정규화 비중)=3.67%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지자체수행보조사업수(LAF_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=3.63%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1153,24 +1153,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SBAT_BDTR_CRCD_EXE_CNT</t>
+          <t>SECT_CD</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>보조금전용신용카드집행건수</t>
+          <t>부문코드</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.0365357161740591</v>
+        <v>0.0351758793969894</v>
       </c>
       <c r="F21" t="n">
-        <v>0.002478701461752442</v>
+        <v>0.0001645561685055807</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>변수 의미: 보조금전용신용카드집행건수(SBAT_BDTR_CRCD_EXE_CNT). 기여도(정규화 비중)=3.65%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.52%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1203,10 +1203,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.2770684556012389</v>
+        <v>0.2562100699289994</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0551125459600037</v>
+        <v>0.08751776161818792</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=27.71%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=25.62%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1225,24 +1225,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.1703274904421835</v>
+        <v>0.1949562418037012</v>
       </c>
       <c r="F23" t="n">
-        <v>0.03388036947358997</v>
+        <v>0.06659431419257783</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=17.03%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=19.50%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1261,24 +1261,24 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>THY_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>부서코드</t>
+          <t>당해년도수행보조사업수</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.1166684700281321</v>
+        <v>0.1093935790725324</v>
       </c>
       <c r="F24" t="n">
-        <v>0.02320688727468401</v>
+        <v>0.03736731026412576</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=11.67%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=10.94%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1297,24 +1297,24 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>당해년도수행보조사업수</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.1080844694510566</v>
+        <v>0.0834101188678308</v>
       </c>
       <c r="F25" t="n">
-        <v>0.02149941709263758</v>
+        <v>0.02849172517552673</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=10.81%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=8.34%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1333,24 +1333,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>BIZ_ENFC_ZON_DV_CD</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>지방자치단체코드</t>
+          <t>사업시행지역구분코드</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.09138534227800571</v>
+        <v>0.07228800501623002</v>
       </c>
       <c r="F26" t="n">
-        <v>0.01817774190655552</v>
+        <v>0.02469256728518898</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=9.14%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 사업시행지역구분코드(BIZ_ENFC_ZON_DV_CD). 기여도(정규화 비중)=7.23%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1369,24 +1369,24 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.06511938252903433</v>
+        <v>0.07008575765338301</v>
       </c>
       <c r="F27" t="n">
-        <v>0.01295309837682734</v>
+        <v>0.02394031051487805</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.51%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=7.01%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1405,24 +1405,24 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BIZ_ENFC_ZON_DV_CD</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>사업시행지역구분코드</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.06332503787059059</v>
+        <v>0.06775733986870594</v>
       </c>
       <c r="F28" t="n">
-        <v>0.01259617971482385</v>
+        <v>0.02314495570043462</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>변수 의미: 사업시행지역구분코드(BIZ_ENFC_ZON_DV_CD). 기여도(정규화 비중)=6.33%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.78%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1441,24 +1441,24 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.040269061530693</v>
+        <v>0.05602349063853686</v>
       </c>
       <c r="F29" t="n">
-        <v>0.008010043942247358</v>
+        <v>0.01913683759612173</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=4.03%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=5.60%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1477,24 +1477,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>RPRSV_DSCRD_YN</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>보조사업자설립년수</t>
+          <t>대표자불일치여부</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.02744716150905338</v>
+        <v>0.03345427851547132</v>
       </c>
       <c r="F30" t="n">
-        <v>0.00545960003587137</v>
+        <v>0.01142751170177209</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=2.74%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자불일치여부(RPRSV_DSCRD_YN). 기여도(정규화 비중)=3.35%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1513,24 +1513,24 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>기관유형코드</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.01709586669552097</v>
+        <v>0.0253984882489458</v>
       </c>
       <c r="F31" t="n">
-        <v>0.00340059187516828</v>
+        <v>0.008675766883985359</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=1.71%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=2.54%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1549,24 +1549,24 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>RPRSV_AGGP_DV_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>대표자연령대구분코드</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.2989836767503042</v>
+        <v>0.1725924154968874</v>
       </c>
       <c r="F32" t="n">
-        <v>0.06737871042955795</v>
+        <v>0.03959796054831155</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=29.90%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=17.26%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1585,24 +1585,24 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>지방자치단체코드</t>
+          <t>대표자연령대구분코드</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.1900691609165165</v>
+        <v>0.1514851372428482</v>
       </c>
       <c r="F33" t="n">
-        <v>0.04283382656264023</v>
+        <v>0.03475530758943485</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=19.01%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=15.15%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1621,24 +1621,24 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>보조사업자설립년수</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.1094318299389545</v>
+        <v>0.1492537313432844</v>
       </c>
       <c r="F34" t="n">
-        <v>0.02466146533943159</v>
+        <v>0.03424335506519549</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=10.94%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=14.93%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1657,24 +1657,24 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.09961877929788324</v>
+        <v>0.1108872115395569</v>
       </c>
       <c r="F35" t="n">
-        <v>0.02245000448390294</v>
+        <v>0.02544090605148774</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=9.96%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=11.09%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1693,24 +1693,24 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>부서코드</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.0671473708505427</v>
+        <v>0.1016428156699347</v>
       </c>
       <c r="F36" t="n">
-        <v>0.01513227513227527</v>
+        <v>0.02331995987963886</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.71%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=10.16%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1729,24 +1729,24 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_DSCRD_YN</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>대표자불일치여부</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.04746555881861263</v>
+        <v>0.07307854321072019</v>
       </c>
       <c r="F37" t="n">
-        <v>0.01069679849340871</v>
+        <v>0.01676644516883979</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=4.75%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자불일치여부(RPRSV_DSCRD_YN). 기여도(정규화 비중)=7.31%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1779,10 +1779,10 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.03771617760586961</v>
+        <v>0.05602422669262386</v>
       </c>
       <c r="F38" t="n">
-        <v>0.008499686126804851</v>
+        <v>0.01285366516215303</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=3.77%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=5.60%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1801,24 +1801,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.03252711919712811</v>
+        <v>0.04550474173753693</v>
       </c>
       <c r="F39" t="n">
-        <v>0.007330284279436938</v>
+        <v>0.01044017469073888</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=3.25%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=4.55%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1837,24 +1837,24 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>BIZ_ENFC_ZON_DV_CD</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>당해년도수행보조사업수</t>
+          <t>사업시행지역구분코드</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.01931571281904346</v>
+        <v>0.02871227387092019</v>
       </c>
       <c r="F40" t="n">
-        <v>0.004352972827549206</v>
+        <v>0.006587470745570034</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=1.93%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 사업시행지역구분코드(BIZ_ENFC_ZON_DV_CD). 기여도(정규화 비중)=2.87%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1873,24 +1873,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BIZ_MDCN</t>
+          <t>THY_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>사업개월수</t>
+          <t>당해년도수행보조사업수</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.01564676201163554</v>
+        <v>0.02771041816091179</v>
       </c>
       <c r="F41" t="n">
-        <v>0.003526141153259887</v>
+        <v>0.006357614510197229</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>변수 의미: 사업개월수(BIZ_MDCN). 기여도(정규화 비중)=1.56%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=2.77%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1923,10 +1923,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.07123498568589968</v>
+        <v>0.0699099314364416</v>
       </c>
       <c r="F42" t="n">
-        <v>0.07123498568589968</v>
+        <v>0.0699099314364416</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=7.12%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=6.99%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1959,10 +1959,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.06438996081869364</v>
+        <v>0.06522771266272298</v>
       </c>
       <c r="F43" t="n">
-        <v>0.06438996081869364</v>
+        <v>0.06522771266272298</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.44%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.52%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1995,10 +1995,10 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.05839048873031386</v>
+        <v>0.06257466028351776</v>
       </c>
       <c r="F44" t="n">
-        <v>0.05839048873031386</v>
+        <v>0.06257466028351776</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=5.84%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.26%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2031,10 +2031,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.05427018714487944</v>
+        <v>0.05371746488869882</v>
       </c>
       <c r="F45" t="n">
-        <v>0.05427018714487944</v>
+        <v>0.05371746488869882</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=5.43%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=5.37%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2053,24 +2053,24 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.05358114621860463</v>
+        <v>0.05359413285871334</v>
       </c>
       <c r="F46" t="n">
-        <v>0.05358114621860463</v>
+        <v>0.05359413285871334</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=5.36%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=5.36%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2089,24 +2089,24 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.05098330684009479</v>
+        <v>0.05314864471147066</v>
       </c>
       <c r="F47" t="n">
-        <v>0.05098330684009479</v>
+        <v>0.05314864471147066</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=5.10%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=5.31%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2139,10 +2139,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.04893369782155989</v>
+        <v>0.05015250059614454</v>
       </c>
       <c r="F48" t="n">
-        <v>0.04893369782155989</v>
+        <v>0.05015250059614454</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=4.89%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=5.02%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2175,10 +2175,10 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.04303240847945023</v>
+        <v>0.04274640347258525</v>
       </c>
       <c r="F49" t="n">
-        <v>0.04303240847945023</v>
+        <v>0.04274640347258525</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.30%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.27%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2211,10 +2211,10 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.03644836213775499</v>
+        <v>0.03684917303412914</v>
       </c>
       <c r="F50" t="n">
-        <v>0.03644836213775499</v>
+        <v>0.03684917303412914</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.64%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.68%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2247,10 +2247,10 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.02993899235451626</v>
+        <v>0.02912809723430759</v>
       </c>
       <c r="F51" t="n">
-        <v>0.02993899235451626</v>
+        <v>0.02912809723430759</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>변수 의미: 사업비보조금금액(BIZCT_SBAT_AMT). 기여도(정규화 비중)=2.99%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 사업비보조금금액(BIZCT_SBAT_AMT). 기여도(정규화 비중)=2.91%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -2325,24 +2325,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>부서코드</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.06671461789117154</v>
+        <v>0.0720834366819162</v>
       </c>
       <c r="F2" t="n">
-        <v>6.671461789117155</v>
+        <v>7.208343668191625</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.67%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=7.21%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2361,24 +2361,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.06495441989195058</v>
+        <v>0.06054513955043873</v>
       </c>
       <c r="F3" t="n">
-        <v>6.495441989195059</v>
+        <v>6.054513955043876</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.50%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.05%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2397,24 +2397,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>기관유형코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.05547755973096497</v>
+        <v>0.05896145497730271</v>
       </c>
       <c r="F4" t="n">
-        <v>5.547755973096498</v>
+        <v>5.896145497730275</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=5.55%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=5.90%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2433,24 +2433,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>LAF_CPRN_AID_BIZCT_RT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>보조사업자설립년수</t>
+          <t>지자체대비보조사업금액비율</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.05417814811546744</v>
+        <v>0.05096941996978932</v>
       </c>
       <c r="F5" t="n">
-        <v>5.417814811546745</v>
+        <v>5.096941996978935</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=5.42%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 지자체대비보조사업금액비율(LAF_CPRN_AID_BIZCT_RT). 기여도(정규화 비중)=5.10%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2469,24 +2469,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>RPRSV_AGGP_DV_CD</t>
+          <t>SECT_CD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대표자연령대구분코드</t>
+          <t>부문코드</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.05058522443296955</v>
+        <v>0.04933380106314258</v>
       </c>
       <c r="F6" t="n">
-        <v>5.058522443296956</v>
+        <v>4.933380106314261</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2495,7 +2495,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=5.06%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=4.93%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2505,24 +2505,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>대표자연령대구분코드</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.04458071949171321</v>
+        <v>0.04914549675775322</v>
       </c>
       <c r="F7" t="n">
-        <v>4.458071949171321</v>
+        <v>4.914549675775325</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=4.46%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=4.91%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2541,24 +2541,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>INST_TY_CD</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>기관유형코드</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.04060187085898578</v>
+        <v>0.04751753225903853</v>
       </c>
       <c r="F8" t="n">
-        <v>4.060187085898579</v>
+        <v>4.751753225903856</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=4.06%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=4.75%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2577,24 +2577,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>지방자치단체코드</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.03611816776722611</v>
+        <v>0.04720868290349021</v>
       </c>
       <c r="F9" t="n">
-        <v>3.611816776722611</v>
+        <v>4.720868290349023</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=3.61%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.72%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2613,24 +2613,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SECT_CD</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>부문코드</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.03477271178468273</v>
+        <v>0.04484785765179874</v>
       </c>
       <c r="F10" t="n">
-        <v>3.477271178468274</v>
+        <v>4.484785765179876</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.48%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=4.48%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2649,24 +2649,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>catboost_v1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LBST_PLAN_RT</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>인건비계획비율</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.0344039068366</v>
+        <v>0.03747459357124595</v>
       </c>
       <c r="F11" t="n">
-        <v>3.44039068366</v>
+        <v>3.747459357124598</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>변수 의미: 인건비계획비율(LBST_PLAN_RT). 기여도(정규화 비중)=3.44%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=3.75%. 측정방법: CatBoost 예측값 변화에 대한 기여도(PredictionValuesChange)입니다. 값이 클수록 위험도 점수에 미치는 영향이 큽니다.</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2755,10 +2755,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.2770684556012389</v>
+        <v>0.2562100699289994</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0551125459600037</v>
+        <v>0.08751776161818792</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=27.71%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=25.62%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2777,24 +2777,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.1703274904421835</v>
+        <v>0.1949562418037012</v>
       </c>
       <c r="F3" t="n">
-        <v>0.03388036947358997</v>
+        <v>0.06659431419257783</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2803,7 +2803,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=17.03%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=19.50%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2813,24 +2813,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>THY_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>부서코드</t>
+          <t>당해년도수행보조사업수</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.1166684700281321</v>
+        <v>0.1093935790725324</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02320688727468401</v>
+        <v>0.03736731026412576</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=11.67%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=10.94%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2849,24 +2849,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>당해년도수행보조사업수</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.1080844694510566</v>
+        <v>0.0834101188678308</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02149941709263758</v>
+        <v>0.02849172517552673</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=10.81%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=8.34%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2885,24 +2885,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>BIZ_ENFC_ZON_DV_CD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>지방자치단체코드</t>
+          <t>사업시행지역구분코드</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.09138534227800571</v>
+        <v>0.07228800501623002</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01817774190655552</v>
+        <v>0.02469256728518898</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -2911,7 +2911,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=9.14%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 사업시행지역구분코드(BIZ_ENFC_ZON_DV_CD). 기여도(정규화 비중)=7.23%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2921,24 +2921,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.06511938252903433</v>
+        <v>0.07008575765338301</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01295309837682734</v>
+        <v>0.02394031051487805</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.51%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=7.01%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2957,24 +2957,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BIZ_ENFC_ZON_DV_CD</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>사업시행지역구분코드</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.06332503787059059</v>
+        <v>0.06775733986870594</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01259617971482385</v>
+        <v>0.02314495570043462</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>변수 의미: 사업시행지역구분코드(BIZ_ENFC_ZON_DV_CD). 기여도(정규화 비중)=6.33%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.78%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -2993,24 +2993,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.040269061530693</v>
+        <v>0.05602349063853686</v>
       </c>
       <c r="F9" t="n">
-        <v>0.008010043942247358</v>
+        <v>0.01913683759612173</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=4.03%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=5.60%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3029,24 +3029,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>RPRSV_DSCRD_YN</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>보조사업자설립년수</t>
+          <t>대표자불일치여부</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.02744716150905338</v>
+        <v>0.03345427851547132</v>
       </c>
       <c r="F10" t="n">
-        <v>0.00545960003587137</v>
+        <v>0.01142751170177209</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=2.74%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자불일치여부(RPRSV_DSCRD_YN). 기여도(정규화 비중)=3.35%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3065,24 +3065,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>easy_ensemble</t>
+          <t>easy_ensemble_v1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>기관유형코드</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.01709586669552097</v>
+        <v>0.0253984882489458</v>
       </c>
       <c r="F11" t="n">
-        <v>0.00340059187516828</v>
+        <v>0.008675766883985359</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=1.71%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=2.54%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3157,24 +3157,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RPRSV_AGGP_DV_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>대표자연령대구분코드</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.2989836767503042</v>
+        <v>0.1725924154968874</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06737871042955795</v>
+        <v>0.03959796054831155</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=29.90%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=17.26%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3193,24 +3193,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>지방자치단체코드</t>
+          <t>대표자연령대구분코드</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.1900691609165165</v>
+        <v>0.1514851372428482</v>
       </c>
       <c r="F3" t="n">
-        <v>0.04283382656264023</v>
+        <v>0.03475530758943485</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=19.01%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=15.15%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3229,24 +3229,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>보조사업자설립년수</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.1094318299389545</v>
+        <v>0.1492537313432844</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02466146533943159</v>
+        <v>0.03424335506519549</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=10.94%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=14.93%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3265,24 +3265,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.09961877929788324</v>
+        <v>0.1108872115395569</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02245000448390294</v>
+        <v>0.02544090605148774</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=9.96%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=11.09%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3301,24 +3301,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>부서코드</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.0671473708505427</v>
+        <v>0.1016428156699347</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01513227513227527</v>
+        <v>0.02331995987963886</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.71%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=10.16%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3337,24 +3337,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_DSCRD_YN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>대표자불일치여부</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.04746555881861263</v>
+        <v>0.07307854321072019</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01069679849340871</v>
+        <v>0.01676644516883979</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=4.75%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자불일치여부(RPRSV_DSCRD_YN). 기여도(정규화 비중)=7.31%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3387,10 +3387,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.03771617760586961</v>
+        <v>0.05602422669262386</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008499686126804851</v>
+        <v>0.01285366516215303</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=3.77%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=5.60%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3409,24 +3409,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.03252711919712811</v>
+        <v>0.04550474173753693</v>
       </c>
       <c r="F9" t="n">
-        <v>0.007330284279436938</v>
+        <v>0.01044017469073888</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=3.25%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=4.55%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3445,24 +3445,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>BIZ_ENFC_ZON_DV_CD</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>당해년도수행보조사업수</t>
+          <t>사업시행지역구분코드</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.01931571281904346</v>
+        <v>0.02871227387092019</v>
       </c>
       <c r="F10" t="n">
-        <v>0.004352972827549206</v>
+        <v>0.006587470745570034</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=1.93%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 사업시행지역구분코드(BIZ_ENFC_ZON_DV_CD). 기여도(정규화 비중)=2.87%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3481,24 +3481,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>gradient_boosting</t>
+          <t>gradient_boosting_v1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BIZ_MDCN</t>
+          <t>THY_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>사업개월수</t>
+          <t>당해년도수행보조사업수</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.01564676201163554</v>
+        <v>0.02771041816091179</v>
       </c>
       <c r="F11" t="n">
-        <v>0.003526141153259887</v>
+        <v>0.006357614510197229</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>변수 의미: 사업개월수(BIZ_MDCN). 기여도(정규화 비중)=1.56%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=2.77%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -3573,7 +3573,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3587,10 +3587,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.07123498568589968</v>
+        <v>0.0699099314364416</v>
       </c>
       <c r="F2" t="n">
-        <v>0.07123498568589968</v>
+        <v>0.0699099314364416</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=7.12%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=6.99%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3623,10 +3623,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.06438996081869364</v>
+        <v>0.06522771266272298</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06438996081869364</v>
+        <v>0.06522771266272298</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.44%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=6.52%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3659,10 +3659,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.05839048873031386</v>
+        <v>0.06257466028351776</v>
       </c>
       <c r="F4" t="n">
-        <v>0.05839048873031386</v>
+        <v>0.06257466028351776</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=5.84%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=6.26%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3695,10 +3695,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.05427018714487944</v>
+        <v>0.05371746488869882</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05427018714487944</v>
+        <v>0.05371746488869882</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=5.43%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=5.37%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3717,24 +3717,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.05358114621860463</v>
+        <v>0.05359413285871334</v>
       </c>
       <c r="F6" t="n">
-        <v>0.05358114621860463</v>
+        <v>0.05359413285871334</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=5.36%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=5.36%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3753,24 +3753,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>대표자세대구분코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.05098330684009479</v>
+        <v>0.05314864471147066</v>
       </c>
       <c r="F7" t="n">
-        <v>0.05098330684009479</v>
+        <v>0.05314864471147066</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=5.10%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=5.31%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3803,10 +3803,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.04893369782155989</v>
+        <v>0.05015250059614454</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04893369782155989</v>
+        <v>0.05015250059614454</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=4.89%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=5.02%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3825,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3839,10 +3839,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.04303240847945023</v>
+        <v>0.04274640347258525</v>
       </c>
       <c r="F9" t="n">
-        <v>0.04303240847945023</v>
+        <v>0.04274640347258525</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.30%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.27%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3861,7 +3861,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3875,10 +3875,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.03644836213775499</v>
+        <v>0.03684917303412914</v>
       </c>
       <c r="F10" t="n">
-        <v>0.03644836213775499</v>
+        <v>0.03684917303412914</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.64%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.68%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>random_forest</t>
+          <t>random_forest_v1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3911,10 +3911,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.02993899235451626</v>
+        <v>0.02912809723430759</v>
       </c>
       <c r="F11" t="n">
-        <v>0.02993899235451626</v>
+        <v>0.02912809723430759</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>변수 의미: 사업비보조금금액(BIZCT_SBAT_AMT). 기여도(정규화 비중)=2.99%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
+          <t>변수 의미: 사업비보조금금액(BIZCT_SBAT_AMT). 기여도(정규화 비중)=2.91%. 측정방법: 트리 분할 시 불순도(오분류)를 줄이는 데 기여한 상대 비중입니다. 값이 클수록 모델이 예측에 더 자주·강하게 사용한 변수입니다.</t>
         </is>
       </c>
     </row>
@@ -3989,24 +3989,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MBR_NUM</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>회원수</t>
+          <t>지방자치단체코드</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.1027335695024538</v>
+        <v>0.1781127861529395</v>
       </c>
       <c r="F2" t="n">
-        <v>0.006969778495202472</v>
+        <v>0.0008332288532263421</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -4015,7 +4015,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=10.27%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지방자치단체코드(LAF_CD). 기여도(정규화 비중)=17.81%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4025,24 +4025,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>AID_BZR_CAP_CD</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>기관유형코드</t>
+          <t>보조사업자시도코드</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.09652091154231966</v>
+        <v>0.09715242881070832</v>
       </c>
       <c r="F3" t="n">
-        <v>0.006548291633037551</v>
+        <v>0.0004544884653962522</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>변수 의미: 기관유형코드(INST_TY_CD). 기여도(정규화 비중)=9.65%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=9.72%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4061,24 +4061,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>MBR_NUM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>상근직원수</t>
+          <t>회원수</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.07809443240098939</v>
+        <v>0.09659408151866568</v>
       </c>
       <c r="F4" t="n">
-        <v>0.005298179535467795</v>
+        <v>0.0004518764627214344</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=7.81%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 회원수(MBR_NUM). 기여도(정규화 비중)=9.66%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4097,24 +4097,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BIZ_MDCN</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>사업개월수</t>
+          <t>대표자세대구분코드</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.06968751652302239</v>
+        <v>0.08096035734221936</v>
       </c>
       <c r="F5" t="n">
-        <v>0.00472782710070857</v>
+        <v>0.0003787403878300344</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>변수 의미: 사업개월수(BIZ_MDCN). 기여도(정규화 비중)=6.97%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자세대구분코드(RPRSV_HSHD_DV_CD). 기여도(정규화 비중)=8.10%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4133,24 +4133,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LAF_PFM_AID_BIZ_NUM</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>지자체수행보조사업수</t>
+          <t>부서코드</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.05950933220535835</v>
+        <v>0.07146845337799287</v>
       </c>
       <c r="F6" t="n">
-        <v>0.004037306071204505</v>
+        <v>0.0003343363423604639</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>변수 의미: 지자체수행보조사업수(LAF_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=5.95%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부서코드(DEPT_CD). 기여도(정규화 비중)=7.15%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4169,24 +4169,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>당해년도수행보조사업수</t>
+          <t>보조사업자설립년수</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.05448633215248471</v>
+        <v>0.04578447794526556</v>
       </c>
       <c r="F7" t="n">
-        <v>0.003696529459241427</v>
+        <v>0.0002141842193246202</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>변수 의미: 당해년도수행보조사업수(THY_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=5.45%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 보조사업자설립년수(AID_BZR_FNDN_YS). 기여도(정규화 비중)=4.58%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4205,24 +4205,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AID_BZR_CAP_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>보조사업자시도코드</t>
+          <t>상근직원수</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.04909321630624239</v>
+        <v>0.03852596314907911</v>
       </c>
       <c r="F8" t="n">
-        <v>0.003330642991660082</v>
+        <v>0.0001802281845537101</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>변수 의미: 보조사업자시도코드(AID_BZR_CAP_CD). 기여도(정규화 비중)=4.91%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 상근직원수(FTEP_STF_NUM). 기여도(정규화 비중)=3.85%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4241,24 +4241,24 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LBST_PLAN_RT</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>인건비계획비율</t>
+          <t>대표자연령대구분코드</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.04446676888912223</v>
+        <v>0.03740926856505316</v>
       </c>
       <c r="F9" t="n">
-        <v>0.003016769796430951</v>
+        <v>0.0001750041792043522</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>변수 의미: 인건비계획비율(LBST_PLAN_RT). 기여도(정규화 비중)=4.45%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 대표자연령대구분코드(RPRSV_AGGP_DV_CD). 기여도(정규화 비중)=3.74%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4277,24 +4277,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BIZCT_PYHWY_AMT</t>
+          <t>LAF_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>사업비자부담금액</t>
+          <t>지자체수행보조사업수</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.03666790038597665</v>
+        <v>0.03629257398101535</v>
       </c>
       <c r="F10" t="n">
-        <v>0.002487669267330406</v>
+        <v>0.0001697801738549387</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>변수 의미: 사업비자부담금액(BIZCT_PYHWY_AMT). 기여도(정규화 비중)=3.67%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 지자체수행보조사업수(LAF_PFM_AID_BIZ_NUM). 기여도(정규화 비중)=3.63%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>
@@ -4313,24 +4313,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>stacked_ensemble</t>
+          <t>stacked_ensemble_v1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SBAT_BDTR_CRCD_EXE_CNT</t>
+          <t>SECT_CD</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>보조금전용신용카드집행건수</t>
+          <t>부문코드</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.0365357161740591</v>
+        <v>0.0351758793969894</v>
       </c>
       <c r="F11" t="n">
-        <v>0.002478701461752442</v>
+        <v>0.0001645561685055807</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -4339,7 +4339,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>변수 의미: 보조금전용신용카드집행건수(SBAT_BDTR_CRCD_EXE_CNT). 기여도(정규화 비중)=3.65%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
+          <t>변수 의미: 부문코드(SECT_CD). 기여도(정규화 비중)=3.52%. 측정방법: 해당 변수 값을 무작위로 섞었을 때 ROC-AUC가 얼마나 떨어지는지로 측정했습니다. 하락이 클수록 그 변수가 중요합니다.</t>
         </is>
       </c>
     </row>

</xml_diff>